<commit_message>
Email enviado para os contatos que faltavam
</commit_message>
<xml_diff>
--- a/Reports/contatos.xlsx
+++ b/Reports/contatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO1\Downloads\Fluxo-da-Comunicacao-Cientifica-Lic-Comp\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15866AD-DC37-45B8-8E54-90354DF7F8C5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAFB246-A592-4020-8D40-71D27E827CFA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{C6D5BA5E-50F0-4F39-A2EF-B634676C8535}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="119">
   <si>
     <t>Nome</t>
   </si>
@@ -301,9 +301,6 @@
   </si>
   <si>
     <t>riuel@uel.br</t>
-  </si>
-  <si>
-    <t>não enviado</t>
   </si>
   <si>
     <t>dspaceuespi4@gmail.com</t>
@@ -394,10 +391,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -423,8 +427,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -739,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D684ADCB-AF66-40B4-815A-350BF8C6BB3D}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="81.42578125" bestFit="1" customWidth="1"/>
@@ -777,16 +782,16 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" t="s">
         <v>117</v>
       </c>
-      <c r="B3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>118</v>
-      </c>
-      <c r="D3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -971,7 +976,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
@@ -985,7 +990,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>48</v>
       </c>
@@ -999,7 +1004,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1009,11 +1014,11 @@
       <c r="C19" t="s">
         <v>53</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -1027,7 +1032,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1041,7 +1046,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1055,7 +1060,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -1065,79 +1070,67 @@
       <c r="C23" t="s">
         <v>67</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D24" t="s">
         <v>90</v>
       </c>
-      <c r="E24" t="s">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" t="s">
         <v>107</v>
       </c>
-      <c r="B25" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" t="s">
-        <v>95</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="C26" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" t="s">
         <v>92</v>
       </c>
-      <c r="E25" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" t="s">
         <v>109</v>
       </c>
-      <c r="B26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>97</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>93</v>
       </c>
-      <c r="E26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" t="s">
-        <v>110</v>
-      </c>
-      <c r="C27" t="s">
-        <v>98</v>
-      </c>
-      <c r="D27" t="s">
-        <v>94</v>
-      </c>
-      <c r="E27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>63</v>
       </c>
@@ -1145,44 +1138,38 @@
         <v>64</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" t="s">
+        <v>111</v>
+      </c>
+      <c r="C29" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" t="s">
         <v>113</v>
       </c>
-      <c r="B29" t="s">
-        <v>112</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" t="s">
         <v>101</v>
-      </c>
-      <c r="D29" t="s">
-        <v>100</v>
-      </c>
-      <c r="E29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" t="s">
-        <v>114</v>
-      </c>
-      <c r="C30" t="s">
-        <v>103</v>
-      </c>
-      <c r="D30" t="s">
-        <v>102</v>
-      </c>
-      <c r="E30" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1196,8 +1183,14 @@
     <hyperlink ref="C3" r:id="rId6" xr:uid="{04EB3C13-602C-4BBD-99BA-9894B1424F46}"/>
     <hyperlink ref="D3" r:id="rId7" xr:uid="{390AB778-8D6C-4A22-BD9B-67EC2F6485CA}"/>
     <hyperlink ref="D28" r:id="rId8" display="mailto:diretoria-samaro@ifba.edu.br" xr:uid="{B8386735-4C4E-4127-B84C-BBFAF7D61918}"/>
+    <hyperlink ref="C24" r:id="rId9" xr:uid="{B0C3B9C2-FB6C-4E67-933A-64602508911C}"/>
+    <hyperlink ref="C25" r:id="rId10" xr:uid="{F8FD96A1-3990-4F6F-97A5-985F0C1F619B}"/>
+    <hyperlink ref="C26" r:id="rId11" xr:uid="{9BF22398-1440-40C9-B9E6-24CC616A7843}"/>
+    <hyperlink ref="C27" r:id="rId12" xr:uid="{75A85D7E-5FD5-4EA4-8D3E-5051DFEAAFC8}"/>
+    <hyperlink ref="C29" r:id="rId13" xr:uid="{EB5DA9C4-40F2-4CAB-8D8C-A2042C6C895D}"/>
+    <hyperlink ref="C30" r:id="rId14" xr:uid="{58FEC2C7-BA20-46D5-B40A-9414AE634E40}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>